<commit_message>
FHS anbd Cognitive test scoring
- added scoring for cognitive tests
- added scoring for FHS
- built infrastructure to share processed output with the RU
- updated VPID renaming audit
- ensured no confidential data is  loaded on GitHub
-- yet to be put otgether so it runs
</commit_message>
<xml_diff>
--- a/information/2025-11-10_Target_Sample_Size_Projects.xlsx
+++ b/information/2025-11-10_Target_Sample_Size_Projects.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Wilken Arbeitsordner\Clinical_Backbone_RU5389\information\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Wilken_Arbeitsordner\Clinical_Backbone_RU5389\information\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1836EE8B-BF94-44DA-AB5A-BA18BAECC95F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FABA4EA-B98F-4970-A2B5-C8CA404EC893}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6750" yWindow="4410" windowWidth="19185" windowHeight="10065" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Vanilla" sheetId="1" r:id="rId1"/>
@@ -543,7 +543,7 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>64</v>
+        <v>44</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
cogntiiver tests, fixes to the pipeline, new ID fixes
</commit_message>
<xml_diff>
--- a/information/2025-11-10_Target_Sample_Size_Projects.xlsx
+++ b/information/2025-11-10_Target_Sample_Size_Projects.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Wilken_Arbeitsordner\Clinical_Backbone_RU5389\information\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FABA4EA-B98F-4970-A2B5-C8CA404EC893}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{419B80BA-6399-4AD5-8084-B46E613795F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -490,7 +490,7 @@
         <v>0</v>
       </c>
       <c r="B2">
-        <v>120</v>
+        <v>102</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>